<commit_message>
docs: developer start guide, task-cycle and branch rules, story refs in task files
</commit_message>
<xml_diff>
--- a/docs/bmad/VulnMart-Tracker.xlsx
+++ b/docs/bmad/VulnMart-Tracker.xlsx
@@ -963,7 +963,7 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Milestone engine and evidence capture</t>
+          <t>Milestone engine, evidence capture and sharing signal</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Time metrics, event log and sharing signal</t>
+          <t>Time metrics and event log</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">

</xml_diff>